<commit_message>
1.	Report name based on Time and Date 2.	Improvement in logic for assertion Toast message. 3.	Implement Multi organization in current flow 4. Improvement in report 5. Screenshots with screenname
</commit_message>
<xml_diff>
--- a/ResourcesPK/DistributorShuffling1.xlsx
+++ b/ResourcesPK/DistributorShuffling1.xlsx
@@ -5,16 +5,16 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\ExcelGenerator\ResourcesPK\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Huzaifa\JAR\ResourcesPK\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930"/>
   </bookViews>
   <sheets>
     <sheet name="Excel Template" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913" concurrentManualCount="8"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -48,9 +48,6 @@
     <t>Hvhchch</t>
   </si>
   <si>
-    <t>6180128</t>
-  </si>
-  <si>
     <t>C0154186809</t>
   </si>
   <si>
@@ -61,6 +58,9 @@
   </si>
   <si>
     <t>C00020</t>
+  </si>
+  <si>
+    <t>15178537</t>
   </si>
 </sst>
 </file>
@@ -381,18 +381,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -415,18 +415,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>13</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
@@ -435,7 +435,7 @@
         <v>8</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>